<commit_message>
UPDATE: HP Icon color change & Location name
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8C68D5-02BF-4B27-A9B2-FCAB3408D3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CC9A9D-2543-4B35-841C-D59D5700B59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
   <si>
     <t>key</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -608,6 +608,96 @@
   </si>
   <si>
     <t>Night fog obscures the way, wasting time and energy.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_2</t>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_3</t>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_4</t>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_5</t>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_6</t>
+  </si>
+  <si>
+    <t>EVENT_LOCATION_7</t>
+  </si>
+  <si>
+    <t>EVENT_ARRIVE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已到达</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Visiting</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>盘旋城郊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>笙阡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>峪望</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outer Circling</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Promoton</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>婺​治</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>尚​郢</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>蓬丈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>畈馈</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feedberg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Addicthorp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Incremont</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Materiar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Desirough</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -615,7 +705,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -629,6 +719,12 @@
       <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -654,8 +750,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -972,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E6B57D-D8BE-4224-A2B7-F664CEDC5AD4}">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24.125" customWidth="1"/>
@@ -1597,6 +1696,94 @@
         <v>58</v>
       </c>
     </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>175</v>
+      </c>
+      <c r="B58" t="s">
+        <v>177</v>
+      </c>
+      <c r="C58" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>168</v>
+      </c>
+      <c r="B59" t="s">
+        <v>181</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>169</v>
+      </c>
+      <c r="B60" t="s">
+        <v>182</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>170</v>
+      </c>
+      <c r="B61" t="s">
+        <v>191</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>171</v>
+      </c>
+      <c r="B62" t="s">
+        <v>190</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>172</v>
+      </c>
+      <c r="B63" t="s">
+        <v>187</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>173</v>
+      </c>
+      <c r="B64" t="s">
+        <v>189</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>174</v>
+      </c>
+      <c r="B65" t="s">
+        <v>188</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
NEW: Location UI added
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CC9A9D-2543-4B35-841C-D59D5700B59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE075E1E-18AE-4ADA-94E7-95815037AF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
+    <workbookView xWindow="6105" yWindow="345" windowWidth="21780" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -641,10 +641,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Visiting</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>盘旋城郊</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -698,6 +694,10 @@
   </si>
   <si>
     <t>Desirough</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Now Visiting</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1701,7 +1701,7 @@
         <v>175</v>
       </c>
       <c r="B58" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="C58" t="s">
         <v>176</v>
@@ -1712,10 +1712,10 @@
         <v>168</v>
       </c>
       <c r="B59" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1723,10 +1723,10 @@
         <v>169</v>
       </c>
       <c r="B60" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1734,10 +1734,10 @@
         <v>170</v>
       </c>
       <c r="B61" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1745,10 +1745,10 @@
         <v>171</v>
       </c>
       <c r="B62" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1756,10 +1756,10 @@
         <v>172</v>
       </c>
       <c r="B63" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1767,10 +1767,10 @@
         <v>173</v>
       </c>
       <c r="B64" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1778,10 +1778,10 @@
         <v>174</v>
       </c>
       <c r="B65" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Score UI adjusted
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE075E1E-18AE-4ADA-94E7-95815037AF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E01308D-459A-438C-934F-68B5A5B1E907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6105" yWindow="345" windowWidth="21780" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
@@ -213,26 +213,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>adventure score</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>final score</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>冒险圆满结束了。\n度过了有收获的60天。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冒险失败了。\n会是人生中难忘的60天。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Adventure Failed.\nIt will be an unforgettable 60 days of your life.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Adventure Succeeded.\n60 days well spent.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -698,6 +682,22 @@
   </si>
   <si>
     <t>Now Visiting</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Adventure Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Final Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冒险失败了。\n要是在城里多盘旋一下的话…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Adventure failed. \nMight as well have circled around the city for a little longer...</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1093,13 +1093,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1107,10 +1107,10 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1118,10 +1118,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1129,10 +1129,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1140,10 +1140,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1151,10 +1151,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1162,10 +1162,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1173,10 +1173,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1184,10 +1184,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1195,10 +1195,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1206,10 +1206,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1217,10 +1217,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1228,10 +1228,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1239,10 +1239,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1250,10 +1250,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1261,10 +1261,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1272,10 +1272,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C18" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1283,10 +1283,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1294,10 +1294,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1305,10 +1305,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1316,10 +1316,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1327,10 +1327,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1338,10 +1338,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1349,10 +1349,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1360,10 +1360,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1371,10 +1371,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1382,10 +1382,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1393,10 +1393,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C29" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1404,10 +1404,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1415,10 +1415,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1426,10 +1426,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1437,10 +1437,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C33" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1448,10 +1448,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C34" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1459,10 +1459,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C35" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1470,10 +1470,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C36" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1481,10 +1481,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C37" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1492,10 +1492,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C38" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1503,10 +1503,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1514,10 +1514,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C40" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1525,10 +1525,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C41" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1536,10 +1536,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1547,10 +1547,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C43" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1558,10 +1558,10 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>63</v>
+        <v>191</v>
       </c>
       <c r="C44" t="s">
-        <v>62</v>
+        <v>190</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1569,10 +1569,10 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C45" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1580,10 +1580,10 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C46" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1591,10 +1591,10 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C47" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1602,10 +1602,10 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C48" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1613,10 +1613,10 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C49" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1624,10 +1624,10 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C50" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1635,10 +1635,10 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C51" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1646,10 +1646,10 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C52" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1657,10 +1657,10 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C53" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1668,10 +1668,10 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C54" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1679,7 +1679,7 @@
         <v>55</v>
       </c>
       <c r="B55" t="s">
-        <v>59</v>
+        <v>188</v>
       </c>
       <c r="C55" t="s">
         <v>56</v>
@@ -1690,7 +1690,7 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>60</v>
+        <v>189</v>
       </c>
       <c r="C56" t="s">
         <v>58</v>
@@ -1698,90 +1698,90 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B58" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C58" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B59" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B60" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B61" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B62" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B63" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B64" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B65" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: NEW Events implemented
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E01308D-459A-438C-934F-68B5A5B1E907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B332320-5157-4244-95FB-CCA47D0C48B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6105" yWindow="345" windowWidth="21780" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
+    <workbookView xWindow="6105" yWindow="345" windowWidth="31800" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="186">
   <si>
     <t>key</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -183,12 +183,6 @@
     <t>EVENT_FAILURE_8</t>
   </si>
   <si>
-    <t>EVENT_FAILURE_9</t>
-  </si>
-  <si>
-    <t>EVENT_FAILURE_10</t>
-  </si>
-  <si>
     <t>EVENT_SUCCESS</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -225,376 +219,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>离开了盘旋城。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Left the City of Circling.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>任务罗盘指明隐秘山径，探索效率大幅提升。</t>
-  </si>
-  <si>
-    <t>藏宝图揭示地下洞穴入口，发现珍贵古物。</t>
-  </si>
-  <si>
-    <t>任务日志记录前人经验，顺利解开机关谜题。</t>
-  </si>
-  <si>
-    <t>战斗通行证换取支援，加快关卡推进速度。</t>
-  </si>
-  <si>
-    <t>滑板高速穿越峡谷，节省大量行进时间。</t>
-  </si>
-  <si>
-    <t>钩爪挂住悬崖边稀有矿石，成功采集。</t>
-  </si>
-  <si>
-    <t>跳板助力跃上高台，找到隐藏宝箱。</t>
-  </si>
-  <si>
-    <t>火箭短暂冲刺避开障碍，率先收集资源。</t>
-  </si>
-  <si>
-    <t>传送门直达远方废墟，探索范围扩大。</t>
-  </si>
-  <si>
-    <t>水晶球提前显现路径陷阱，顺利避开危险。</t>
-  </si>
-  <si>
-    <t>钱袋发现额外金币，完成交易更为顺利。</t>
-  </si>
-  <si>
-    <t>天平衡量交易公平，换得珍稀补给。</t>
-  </si>
-  <si>
-    <t>积分券换得隐藏奖励，加快装备升级。</t>
-  </si>
-  <si>
-    <t>会员卡解锁秘密商店，获得稀有物资。</t>
-  </si>
-  <si>
-    <t>四叶草在风中闪耀好运，意外发现珍宝。</t>
-  </si>
-  <si>
-    <t>骰子掷出奇妙点数，触发额外探索机会。</t>
-  </si>
-  <si>
-    <t>山谷回声暴露隐藏通道，获得重要线索。</t>
-  </si>
-  <si>
-    <t>古树下闪烁光点，找到珍贵符文。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>河岸边出现破碎遗迹，拾得历史资料。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>夜空流星划过，发现暗示宝藏的标记。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>风吹落古老卷轴，解开机关提示。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>悬崖石缝中显露稀有草药，可制作强化物品。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>废墟中回响神秘乐声，揭示隐藏路线。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>雨后彩虹照亮裂谷，找到捷径通路。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荒野石堆中隐藏碎片，组合成有用道具。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>岩洞深处闪烁金光，解锁新的探险目标。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荒原沙地露出古代遗迹，获得线索碎片。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>石桥裂缝中发现闪光宝石，增强装备效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>密林小径露出隐秘药草，制作生命补剂。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高塔阴影下藏着古卷，顺利解锁谜题。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>河边废墟里出现闪光碎片，发现隐藏资源。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>山洞回音显现方向，快速穿越险地。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>雪地遗迹中找到储藏箱，收获稀有材料。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>悬崖边闪烁光点，引导安全下行路径。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荒林深处偶现古代符号，推进任务进度。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>沙漠废墟里出现破碎石板，获得重要线索。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>山谷流水旁显露闪光矿石，成功采集。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荒野小丘上藏有神秘宝物，解锁额外探索。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荒林草丛闪烁光芒，发现隐藏补给。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高塔废墟中掉落古代卷轴，推进探险进程。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>罗盘指针失灵，迷失方向延误行进。</t>
-  </si>
-  <si>
-    <t>滑板陷入泥泞，行动速度大幅降低。</t>
-  </si>
-  <si>
-    <t>火箭失控撞向岩壁，损失稀有资源。</t>
-  </si>
-  <si>
-    <t>钩爪断裂，从高台跌落受伤。</t>
-  </si>
-  <si>
-    <t>野兽猛扑，受伤严重影响行动。</t>
-  </si>
-  <si>
-    <t>落石滚落，险些砸中探险路线。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>荆棘划伤，行动受阻且消耗体力。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>陷阱触发，跌入深坑损失补给。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>寒风侵袭，行动迟缓且精神受扰。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>夜间迷雾笼罩，迷路导致时间浪费。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The task compass points to a hidden mountain path, greatly improving exploration efficiency.</t>
-  </si>
-  <si>
-    <t>The treasure map reveals an underground cave entrance, uncovering valuable artifacts.</t>
-  </si>
-  <si>
-    <t>The task log records previous explorers’ experience, unlocking complex mechanisms smoothly.</t>
-  </si>
-  <si>
-    <t>The battle pass grants extra support, accelerating progression through the stage.</t>
-  </si>
-  <si>
-    <t>The skateboard speeds across the canyon, saving significant travel time.</t>
-  </si>
-  <si>
-    <t>The grappling hook secures rare ore on a cliff, allowing successful collection.</t>
-  </si>
-  <si>
-    <t>The rocket dash bypasses obstacles, gaining resources ahead of time.</t>
-  </si>
-  <si>
-    <t>The portal leads directly to a distant ruin, expanding the exploration range.</t>
-  </si>
-  <si>
-    <t>The voucher redeems hidden rewards, accelerating equipment upgrades.</t>
-  </si>
-  <si>
-    <t>The membership card unlocks a secret shop, obtaining rare items.</t>
-  </si>
-  <si>
-    <t>The dice roll produces a perfect result, triggering additional exploration opportunities.</t>
-  </si>
-  <si>
-    <t>The jump pad helps reach a high platform, revealing a hidden chest.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The crystal reveals traps along the path, avoiding danger successfully.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The coin bag contains extra coins, enabling smoother trading.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The balance ensures fair trades, acquiring rare supplies.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The clover shines in the wind, revealing unexpected treasures.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The canyon echoes expose a hidden path, gaining vital clues.</t>
-  </si>
-  <si>
-    <t>A flash of light under an ancient tree reveals valuable runes.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ruins by the river provide historical documents for insight.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A shooting star streaks across the night sky, marking a hidden treasure.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Wind blows down an old scroll, revealing mechanism hints.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Rare herbs appear in cliff crevices, usable for crafting enhancements.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Mysterious music echoes through the ruins, unveiling a hidden route.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A rainbow illuminates the ravine, revealing a shortcut.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Debris in the wilderness conceals fragments that form useful tools.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A golden glimmer deep in the cave unlocks a new exploration target.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Exposed ruins in the desert reveal clue fragments for progress.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Glimmering gemstones appear in stone bridge cracks, enhancing equipment.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Secret herbs appear along forest paths, used for life-restoring remedies.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ancient scrolls in a tall tower unlock puzzle solutions.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Glittering fragments appear in riverside ruins, revealing hidden resources.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Echoes in a cave indicate direction, allowing swift passage.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Storage boxes in snowy ruins contain rare materials.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Flickering lights along the cliff guide a safe descent.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ancient symbols appear deep in the forest, advancing task progress.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Broken stone slabs in desert ruins reveal crucial clues.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Shimmering ore is exposed in a valley stream, collected successfully.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hidden treasures on a wild hill unlock additional exploration.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Flickering lights in the forest grass uncover concealed supplies.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ancient scrolls fall in a tower ruin, pushing the expedition forward.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The compass malfunctions, losing direction and delaying progress.</t>
-  </si>
-  <si>
-    <t>The skateboard gets stuck in mud, severely reducing travel speed.</t>
-  </si>
-  <si>
-    <t>The rocket loses control and hits a rock, losing rare resources.</t>
-  </si>
-  <si>
-    <t>The grappling hook breaks, falling from a high platform and getting injured.</t>
-  </si>
-  <si>
-    <t>A wild beast lunges, causing injury and slowing progress.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Rolling boulders nearly block the path.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Thorns cut arms, restricting movement and draining stamina.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A trap triggers, falling into a pit and losing supplies.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Freezing wind slows movement and weakens endurance.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Night fog obscures the way, wasting time and energy.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EVENT_LOCATION_1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -625,10 +249,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>盘旋城郊</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>笙阡</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -637,10 +257,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Outer Circling</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Promoton</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -661,10 +277,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Feedberg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Addicthorp</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -693,11 +305,375 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冒险失败了。\n要是在城里多盘旋一下的话…</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Adventure failed. \nMight as well have circled around the city for a little longer...</t>
+    <t>冒险失败了。\n要是在城里多停留一下的话…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Adventure failed. \nMight as well have stayed in the city for a little longer...</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>精心搭建的营地被摧毁了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>因为充足的物资感到信心满满。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目前一切进展顺利。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>随手解开了路边的谜题。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>留意到一处隐蔽的捷径。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回忆起了出发前的某个念头。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>背包管理成功。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>打水漂破了个人纪录。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在树下的光点获得了宝贝。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在旅行商人手上淘到了便宜货。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>发现了隐藏的温泉。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>领悟了新的技能。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>巧妙地规避了麻烦的区域。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>娴熟地用树枝和石头搭建了火堆。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>心情舒畅的一天。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>雨下整夜，没有睡好。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一条看似捷径的路没能走通。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>高估了自己的跳跃能力，在小河沟摔得一身淤泥。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在河边坐了一整天，鱼饵都被吃完了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>诸事不顺的一天。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>脚步愈发轻快，原来是背包破了洞。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>发现一处绝景。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>完美用上了一个很冷门的生存技巧。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从很高的地方跳下来，毫发无伤。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在湖里洗了个痛快澡。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>三下五除二补好了磨损的鞋。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>干粮肉变质得恰到好处，别有风味。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>没有上路牌的当，坚定了内心的道路。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>断桥旁刚好停着一尾小船。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>爬上了看似不可能的峭壁。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>找到了一根趁手的木棍。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>还剩很多物资，晚餐奢侈了一把。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>登上一座废弃瞭望塔，掌握了周边信息。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>只用一发石头就击落了鸟窝。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>体会到了传说中的跑步高潮。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>烈日下的湖水透心凉。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在无人的房屋里借宿了一宿。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>趁蜂群外出，采集到了蜂蜜。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>今晚的鱼烤得外酥里嫩，恰到好处。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在背包的角落里翻出额外的物资。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>激动人心的冒险开始了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>路过一棵果树，连吃带拿。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在雨点落下的前一秒躲进了一个洞穴。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>征服了眼前的山丘，到顶才发现爬错了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>找到了前人留下的地图。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>发现了一处得天独厚的扎营点。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>长路的尽头发现一块平整如椅的石头，很舒适。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回顾来时路，感受到了成长。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>离开了斗鎏城。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Left the City of Stayvesant.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>斗鎏城郊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feeling confident with ample supplies.</t>
+  </si>
+  <si>
+    <t>Everything is going smoothly so far.</t>
+  </si>
+  <si>
+    <t>Casually solved a roadside puzzle.</t>
+  </si>
+  <si>
+    <t>Noticed a hidden shortcut.</t>
+  </si>
+  <si>
+    <t>Recalled a thought from before departure.</t>
+  </si>
+  <si>
+    <t>Backpack management succeeded.</t>
+  </si>
+  <si>
+    <t>Discovered a hidden hot spring.</t>
+  </si>
+  <si>
+    <t>Learned a new skill.</t>
+  </si>
+  <si>
+    <t>Bargained well with a traveling merchant.</t>
+  </si>
+  <si>
+    <t>Cleverly avoided a troublesome area.</t>
+  </si>
+  <si>
+    <t>A day of pleasant mood.</t>
+  </si>
+  <si>
+    <t>Skillfully built a campfire with sticks and stones.</t>
+  </si>
+  <si>
+    <t>Discovered a breathtaking view.</t>
+  </si>
+  <si>
+    <t>Found a map left by predecessors.</t>
+  </si>
+  <si>
+    <t>Discovered an excellent campsite.</t>
+  </si>
+  <si>
+    <t>Made perfect use of an obscure survival skill.</t>
+  </si>
+  <si>
+    <t>Jumped from a great height unscathed.</t>
+  </si>
+  <si>
+    <t>Enjoyed a refreshing bath in the lake.</t>
+  </si>
+  <si>
+    <t>Quickly repaired worn shoes.</t>
+  </si>
+  <si>
+    <t>A small boat happened to be moored by the broken bridge.</t>
+  </si>
+  <si>
+    <t>Found a handy stick.</t>
+  </si>
+  <si>
+    <t>With plenty of supplies left, indulged in a lavish dinner.</t>
+  </si>
+  <si>
+    <t>Passed a fruit tree, ate and stocked up.</t>
+  </si>
+  <si>
+    <t>Climbed an abandoned watchtower, surveyed the surroundings.</t>
+  </si>
+  <si>
+    <t>The lake water was cooling under the blazing sun.</t>
+  </si>
+  <si>
+    <t>Ducked into a cave a second before the rain fell.</t>
+  </si>
+  <si>
+    <t>Harvested honey while the bees were away.</t>
+  </si>
+  <si>
+    <t>Stayed overnight in a deserted house.</t>
+  </si>
+  <si>
+    <t>The grilled fish tonight was crispy outside and tender inside.</t>
+  </si>
+  <si>
+    <t>Found extra supplies in a backpack corner.</t>
+  </si>
+  <si>
+    <t>At the end of the road, found a stone smooth as a chair, very comfortable.</t>
+  </si>
+  <si>
+    <t>Looked back on the journey and felt growth.</t>
+  </si>
+  <si>
+    <t>A supposed shortcut led to a dead end.</t>
+  </si>
+  <si>
+    <t>A carefully built camp was destroyed.</t>
+  </si>
+  <si>
+    <t>It rained all night, couldn’t sleep well.</t>
+  </si>
+  <si>
+    <t>Overestimated jumping ability, landed in mud.</t>
+  </si>
+  <si>
+    <t>Sat by the river all day, bait all eaten.</t>
+  </si>
+  <si>
+    <t>A day of constant misfortune.</t>
+  </si>
+  <si>
+    <t>Steps grew lighter—turns out the backpack had a hole.</t>
+  </si>
+  <si>
+    <t>Conquered the hill, only to realize it was the wrong one.</t>
+  </si>
+  <si>
+    <t>An exciting adventure begins.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Broke a personal record on stone skipping.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Found treasure at a shiny spot under the tree.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rations spoiled just right, adding a special flavor.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Didn't fooled by road signs, stayed true to the path.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Climbed an impossible-looking cliff.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outer Stayvesant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feedburg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Experienced the legendary runner's high.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Brought down a bird's nest with just one stone.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -750,12 +726,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1071,13 +1050,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E6B57D-D8BE-4224-A2B7-F664CEDC5AD4}">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24.125" customWidth="1"/>
-    <col min="2" max="2" width="56.875" customWidth="1"/>
+    <col min="2" max="2" width="67.25" customWidth="1"/>
     <col min="3" max="3" width="68.125" customWidth="1"/>
-    <col min="4" max="4" width="20.75" customWidth="1"/>
+    <col min="4" max="4" width="55.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1093,695 +1072,673 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B2" t="s">
-        <v>63</v>
+        <v>59</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>176</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>126</v>
+        <v>178</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="C22" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="C23" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>137</v>
+        <v>179</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>140</v>
+        <v>181</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="C31" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="C33" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="C34" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="C35" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C37" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="C38" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C39" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="C41" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="C42" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="C44" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>43</v>
-      </c>
-      <c r="B45" t="s">
-        <v>154</v>
-      </c>
-      <c r="C45" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>155</v>
+        <v>84</v>
       </c>
       <c r="C46" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B47" t="s">
-        <v>156</v>
-      </c>
-      <c r="C47" t="s">
-        <v>106</v>
+        <v>168</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B48" t="s">
-        <v>157</v>
-      </c>
-      <c r="C48" t="s">
-        <v>107</v>
+        <v>169</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B49" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="C49" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B50" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="C50" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B51" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C51" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B52" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C52" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B53" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C53" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B54" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C54" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>55</v>
-      </c>
-      <c r="B55" t="s">
-        <v>188</v>
-      </c>
-      <c r="C55" t="s">
-        <v>56</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B56" t="s">
-        <v>189</v>
+        <v>81</v>
       </c>
       <c r="C56" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>171</v>
-      </c>
-      <c r="B58" t="s">
-        <v>187</v>
-      </c>
-      <c r="C58" t="s">
-        <v>172</v>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>164</v>
+        <v>67</v>
       </c>
       <c r="B59" t="s">
-        <v>176</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>173</v>
+        <v>80</v>
+      </c>
+      <c r="C59" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>165</v>
+        <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>174</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>166</v>
+        <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>186</v>
+        <v>71</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>175</v>
+        <v>69</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>167</v>
+        <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>185</v>
+        <v>79</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>178</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>168</v>
+        <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>182</v>
+        <v>78</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>169</v>
+        <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>180</v>
+        <v>75</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>170</v>
+        <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>183</v>
+        <v>77</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>179</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>66</v>
+      </c>
+      <c r="B66" t="s">
+        <v>76</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NEW: New Tutorial & Skip button & Failure hide score
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A593FBD6-9EF9-4958-9881-55D4D23D4312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7C664D-99CF-412B-BBF5-1CCEA320C732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6105" yWindow="345" windowWidth="31800" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
@@ -192,10 +192,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冒险点数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>FINAL_SCORE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -706,6 +702,10 @@
   </si>
   <si>
     <t>Used a lockpick to open a chest and found another lockpick inside.</t>
+  </si>
+  <si>
+    <t>冒险得分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1103,13 +1103,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1117,10 +1117,10 @@
         <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1128,10 +1128,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1139,10 +1139,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1150,10 +1150,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1161,10 +1161,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1172,10 +1172,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1183,10 +1183,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1194,10 +1194,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1205,10 +1205,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1216,10 +1216,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1227,10 +1227,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1238,10 +1238,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1249,10 +1249,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1260,10 +1260,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1271,10 +1271,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1282,10 +1282,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1293,10 +1293,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1304,10 +1304,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1315,10 +1315,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1326,10 +1326,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1337,10 +1337,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1348,10 +1348,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1359,10 +1359,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C26" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1370,10 +1370,10 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1381,10 +1381,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1392,10 +1392,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1403,10 +1403,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1414,10 +1414,10 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1425,10 +1425,10 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1436,10 +1436,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1447,10 +1447,10 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1458,10 +1458,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C35" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1469,10 +1469,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1480,10 +1480,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1491,10 +1491,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1502,10 +1502,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1513,10 +1513,10 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1524,10 +1524,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C41" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1535,10 +1535,10 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1546,54 +1546,54 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B44" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C44" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B46" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C46" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B47" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C47" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1601,10 +1601,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1612,10 +1612,10 @@
         <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1623,10 +1623,10 @@
         <v>43</v>
       </c>
       <c r="B52" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1634,10 +1634,10 @@
         <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C53" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1645,10 +1645,10 @@
         <v>45</v>
       </c>
       <c r="B54" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C54" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1656,10 +1656,10 @@
         <v>46</v>
       </c>
       <c r="B55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C55" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1667,10 +1667,10 @@
         <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C56" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1678,10 +1678,10 @@
         <v>48</v>
       </c>
       <c r="B57" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1689,10 +1689,10 @@
         <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C58" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1700,109 +1700,109 @@
         <v>52</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>53</v>
+        <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C61" t="s">
         <v>54</v>
-      </c>
-      <c r="B61" t="s">
-        <v>81</v>
-      </c>
-      <c r="C61" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C63" t="s">
         <v>66</v>
-      </c>
-      <c r="B63" t="s">
-        <v>79</v>
-      </c>
-      <c r="C63" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B64" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B65" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B66" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B68" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B69" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[CHANGE] Ending text adjustment.
逗留，一些文本事件顺序
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\city_of_circling\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7C664D-99CF-412B-BBF5-1CCEA320C732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A70DFB-EAFD-476C-ABFB-F04705874FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6105" yWindow="345" windowWidth="31800" windowHeight="20985" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
+    <workbookView xWindow="-38510" yWindow="1250" windowWidth="38620" windowHeight="21100" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -298,10 +298,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冒险失败了。\n要是在城里多停留一下的话…</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Adventure failed. \nMight as well have stayed in the city for a little longer...</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -434,10 +430,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>登上一座废弃瞭望塔，掌握了周边信息。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>只用一发石头就击落了鸟窝。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -498,18 +490,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>离开了斗鎏城。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Left the City of Stayvesant.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>斗鎏城郊</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Feeling confident with ample supplies.</t>
   </si>
   <si>
@@ -546,9 +530,6 @@
     <t>Skillfully built a campfire with sticks and stones.</t>
   </si>
   <si>
-    <t>Discovered a breathtaking view.</t>
-  </si>
-  <si>
     <t>Found a map left by predecessors.</t>
   </si>
   <si>
@@ -579,9 +560,6 @@
     <t>Passed a fruit tree, ate and stocked up.</t>
   </si>
   <si>
-    <t>Climbed an abandoned watchtower, surveyed the surroundings.</t>
-  </si>
-  <si>
     <t>The lake water was cooling under the blazing sun.</t>
   </si>
   <si>
@@ -705,6 +683,30 @@
   </si>
   <si>
     <t>冒险得分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>离开了逗留城。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>逗留城郊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Discovered a gorgeous view.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Climbed an watchtower, surveyed the surroundings.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>登上了一座瞭望塔，掌握了周边信息。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冒险失败了。\n要是在城里多逗留一下的话…</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -769,7 +771,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -785,9 +787,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -825,7 +827,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -931,7 +933,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1073,7 +1075,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1082,12 +1084,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E6B57D-D8BE-4224-A2B7-F664CEDC5AD4}">
   <dimension ref="A1:C70"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="24.125" customWidth="1"/>
+    <col min="1" max="1" width="24.08203125" customWidth="1"/>
     <col min="2" max="2" width="67.25" customWidth="1"/>
-    <col min="3" max="3" width="68.125" customWidth="1"/>
-    <col min="4" max="4" width="55.375" customWidth="1"/>
+    <col min="3" max="3" width="68.08203125" customWidth="1"/>
+    <col min="4" max="4" width="55.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1106,10 +1108,10 @@
         <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>131</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1128,10 +1130,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1139,10 +1141,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1150,10 +1152,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1161,10 +1163,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1172,10 +1174,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1183,7 +1185,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C10" t="s">
         <v>88</v>
@@ -1194,10 +1196,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1205,10 +1207,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1216,10 +1218,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1227,10 +1229,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1238,10 +1240,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1249,10 +1251,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1260,10 +1262,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1271,10 +1273,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1282,10 +1284,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1293,10 +1295,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1304,10 +1306,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="C21" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1315,10 +1317,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C22" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1326,10 +1328,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1337,10 +1339,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1348,10 +1350,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="C25" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1359,10 +1361,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1370,10 +1372,10 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="C27" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1381,10 +1383,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="C28" t="s">
-        <v>110</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1392,10 +1394,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1403,10 +1405,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1414,7 +1416,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C31" t="s">
         <v>113</v>
@@ -1425,10 +1427,10 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1436,10 +1438,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C33" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1447,10 +1449,10 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="C34" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1458,10 +1460,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
       <c r="C35" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1469,10 +1471,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>182</v>
+        <v>145</v>
       </c>
       <c r="C36" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1480,10 +1482,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1491,10 +1493,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="C38" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1502,10 +1504,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="C39" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1513,10 +1515,10 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="C40" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1524,10 +1526,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="C41" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1535,10 +1537,10 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C42" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1546,54 +1548,54 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C43" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B44" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C44" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B45" t="s">
-        <v>191</v>
+        <v>139</v>
       </c>
       <c r="C45" t="s">
-        <v>188</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B46" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="C46" t="s">
-        <v>189</v>
+        <v>109</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B47" t="s">
-        <v>193</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s">
-        <v>190</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1601,10 +1603,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>194</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1612,10 +1614,10 @@
         <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1623,10 +1625,10 @@
         <v>43</v>
       </c>
       <c r="B52" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1634,10 +1636,10 @@
         <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1645,10 +1647,10 @@
         <v>45</v>
       </c>
       <c r="B54" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1656,10 +1658,10 @@
         <v>46</v>
       </c>
       <c r="B55" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1667,10 +1669,10 @@
         <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C56" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1678,10 +1680,10 @@
         <v>48</v>
       </c>
       <c r="B57" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C57" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1689,10 +1691,10 @@
         <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C58" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1703,7 +1705,7 @@
         <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1733,10 +1735,10 @@
         <v>58</v>
       </c>
       <c r="B64" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1777,7 +1779,7 @@
         <v>62</v>
       </c>
       <c r="B68" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
[CHANGE] minor changes to English ending text
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\city_of_circling\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A70DFB-EAFD-476C-ABFB-F04705874FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7847B7-679C-4BA5-B6B9-DB86E4576B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="1250" windowWidth="38620" windowHeight="21100" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
@@ -548,165 +548,201 @@
     <t>Quickly repaired worn shoes.</t>
   </si>
   <si>
+    <t>Found a handy stick.</t>
+  </si>
+  <si>
+    <t>With plenty of supplies left, indulged in a lavish dinner.</t>
+  </si>
+  <si>
+    <t>Ducked into a cave a second before the rain fell.</t>
+  </si>
+  <si>
+    <t>Harvested honey while the bees were away.</t>
+  </si>
+  <si>
+    <t>Stayed overnight in a deserted house.</t>
+  </si>
+  <si>
+    <t>Found extra supplies in a backpack corner.</t>
+  </si>
+  <si>
+    <t>At the end of the road, found a stone smooth as a chair, very comfortable.</t>
+  </si>
+  <si>
+    <t>Looked back on the journey and felt growth.</t>
+  </si>
+  <si>
+    <t>A supposed shortcut led to a dead end.</t>
+  </si>
+  <si>
+    <t>A carefully built camp was destroyed.</t>
+  </si>
+  <si>
+    <t>It rained all night, couldn’t sleep well.</t>
+  </si>
+  <si>
+    <t>Overestimated jumping ability, landed in mud.</t>
+  </si>
+  <si>
+    <t>Sat by the river all day, bait all eaten.</t>
+  </si>
+  <si>
+    <t>A day of constant misfortune.</t>
+  </si>
+  <si>
+    <t>Steps grew lighter—turns out the backpack had a hole.</t>
+  </si>
+  <si>
+    <t>Conquered the hill, only to realize it was the wrong one.</t>
+  </si>
+  <si>
+    <t>An exciting adventure begins.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Broke a personal record on stone skipping.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rations spoiled just right, adding a special flavor.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Climbed an impossible-looking cliff.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outer Stayvesant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feedburg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Experienced the legendary runner's high.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Brought down a bird's nest with just one stone.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EVENT_SUCCESS_41</t>
+  </si>
+  <si>
+    <t>EVENT_SUCCESS_42</t>
+  </si>
+  <si>
+    <t>EVENT_SUCCESS_43</t>
+  </si>
+  <si>
+    <t>EVENT_SUCCESS_40</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>钓上​了​湖里​最​大​的​鱼。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>​在​地图​上​添​加​了​新​的​标记。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用​撬锁器​打开​了​箱子，​发现​了​撬锁器。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Caught the largest fish in the lake.</t>
+  </si>
+  <si>
+    <t>Added a new marker to the map.</t>
+  </si>
+  <si>
+    <t>Used a lockpick to open a chest and found another lockpick inside.</t>
+  </si>
+  <si>
+    <t>冒险得分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>离开了逗留城。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>逗留城郊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Discovered a gorgeous view.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>登上了一座瞭望塔，掌握了周边信息。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冒险失败了。\n要是在城里多逗留一下的话…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Passed a fruit tree, ate, and stocked up.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Climbed a watchtower, surveyed the surroundings.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tonight's grilled fish was perfectly cooked.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>A small boat happened to be moored by the broken bridge.</t>
-  </si>
-  <si>
-    <t>Found a handy stick.</t>
-  </si>
-  <si>
-    <t>With plenty of supplies left, indulged in a lavish dinner.</t>
-  </si>
-  <si>
-    <t>Passed a fruit tree, ate and stocked up.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>The lake water was cooling under the blazing sun.</t>
-  </si>
-  <si>
-    <t>Ducked into a cave a second before the rain fell.</t>
-  </si>
-  <si>
-    <t>Harvested honey while the bees were away.</t>
-  </si>
-  <si>
-    <t>Stayed overnight in a deserted house.</t>
-  </si>
-  <si>
-    <t>The grilled fish tonight was crispy outside and tender inside.</t>
-  </si>
-  <si>
-    <t>Found extra supplies in a backpack corner.</t>
-  </si>
-  <si>
-    <t>At the end of the road, found a stone smooth as a chair, very comfortable.</t>
-  </si>
-  <si>
-    <t>Looked back on the journey and felt growth.</t>
-  </si>
-  <si>
-    <t>A supposed shortcut led to a dead end.</t>
-  </si>
-  <si>
-    <t>A carefully built camp was destroyed.</t>
-  </si>
-  <si>
-    <t>It rained all night, couldn’t sleep well.</t>
-  </si>
-  <si>
-    <t>Overestimated jumping ability, landed in mud.</t>
-  </si>
-  <si>
-    <t>Sat by the river all day, bait all eaten.</t>
-  </si>
-  <si>
-    <t>A day of constant misfortune.</t>
-  </si>
-  <si>
-    <t>Steps grew lighter—turns out the backpack had a hole.</t>
-  </si>
-  <si>
-    <t>Conquered the hill, only to realize it was the wrong one.</t>
-  </si>
-  <si>
-    <t>An exciting adventure begins.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Broke a personal record on stone skipping.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Found treasure at a shiny spot under the tree.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Rations spoiled just right, adding a special flavor.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Didn't fooled by road signs, stayed true to the path.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Climbed an impossible-looking cliff.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Outer Stayvesant</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Feedburg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Experienced the legendary runner's high.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Brought down a bird's nest with just one stone.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EVENT_SUCCESS_41</t>
-  </si>
-  <si>
-    <t>EVENT_SUCCESS_42</t>
-  </si>
-  <si>
-    <t>EVENT_SUCCESS_43</t>
-  </si>
-  <si>
-    <t>EVENT_SUCCESS_40</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>钓上​了​湖里​最​大​的​鱼。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>​在​地图​上​添​加​了​新​的​标记。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>用​撬锁器​打开​了​箱子，​发现​了​撬锁器。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Caught the largest fish in the lake.</t>
-  </si>
-  <si>
-    <t>Added a new marker to the map.</t>
-  </si>
-  <si>
-    <t>Used a lockpick to open a chest and found another lockpick inside.</t>
-  </si>
-  <si>
-    <t>冒险得分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>离开了逗留城。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>逗留城郊</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Discovered a gorgeous view.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Climbed an watchtower, surveyed the surroundings.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>登上了一座瞭望塔，掌握了周边信息。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>冒险失败了。\n要是在城里多逗留一下的话…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wasn't fooled by road signs, stayed true to the path.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Found treasure at a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>shiny</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>under the tree.</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -714,7 +750,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -733,6 +769,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="等线"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="等线"/>
       <scheme val="minor"/>
     </font>
@@ -1111,7 +1154,7 @@
         <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1130,7 +1173,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C5" t="s">
         <v>121</v>
@@ -1207,10 +1250,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C12" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1218,7 +1261,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="C13" t="s">
         <v>90</v>
@@ -1262,7 +1305,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C17" t="s">
         <v>112</v>
@@ -1284,7 +1327,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C19" t="s">
         <v>89</v>
@@ -1306,10 +1349,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C21" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1339,7 +1382,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>151</v>
+        <v>188</v>
       </c>
       <c r="C24" t="s">
         <v>122</v>
@@ -1350,7 +1393,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C25" t="s">
         <v>103</v>
@@ -1361,7 +1404,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C26" t="s">
         <v>118</v>
@@ -1372,7 +1415,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C27" t="s">
         <v>120</v>
@@ -1383,10 +1426,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C28" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1394,10 +1437,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C29" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1405,7 +1448,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>156</v>
+        <v>190</v>
       </c>
       <c r="C30" t="s">
         <v>119</v>
@@ -1416,7 +1459,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C31" t="s">
         <v>113</v>
@@ -1449,7 +1492,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C34" t="s">
         <v>108</v>
@@ -1460,7 +1503,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C35" t="s">
         <v>128</v>
@@ -1482,7 +1525,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>148</v>
+        <v>191</v>
       </c>
       <c r="C37" t="s">
         <v>110</v>
@@ -1493,7 +1536,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C38" t="s">
         <v>114</v>
@@ -1504,7 +1547,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C39" t="s">
         <v>115</v>
@@ -1515,7 +1558,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="C40" t="s">
         <v>116</v>
@@ -1526,7 +1569,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C41" t="s">
         <v>123</v>
@@ -1537,7 +1580,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C42" t="s">
         <v>117</v>
@@ -1548,7 +1591,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C43" t="s">
         <v>127</v>
@@ -1556,10 +1599,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B44" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C44" t="s">
         <v>111</v>
@@ -1567,7 +1610,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B45" t="s">
         <v>139</v>
@@ -1578,10 +1621,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B46" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="C46" t="s">
         <v>109</v>
@@ -1589,7 +1632,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B47" t="s">
         <v>144</v>
@@ -1606,7 +1649,7 @@
         <v>81</v>
       </c>
       <c r="C50" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1614,7 +1657,7 @@
         <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>98</v>
@@ -1625,7 +1668,7 @@
         <v>43</v>
       </c>
       <c r="B52" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>82</v>
@@ -1636,7 +1679,7 @@
         <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C53" t="s">
         <v>97</v>
@@ -1647,7 +1690,7 @@
         <v>45</v>
       </c>
       <c r="B54" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C54" t="s">
         <v>99</v>
@@ -1658,7 +1701,7 @@
         <v>46</v>
       </c>
       <c r="B55" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C55" t="s">
         <v>100</v>
@@ -1669,7 +1712,7 @@
         <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C56" t="s">
         <v>101</v>
@@ -1680,7 +1723,7 @@
         <v>48</v>
       </c>
       <c r="B57" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C57" t="s">
         <v>102</v>
@@ -1691,7 +1734,7 @@
         <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C58" t="s">
         <v>124</v>
@@ -1705,7 +1748,7 @@
         <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1735,10 +1778,10 @@
         <v>58</v>
       </c>
       <c r="B64" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1779,7 +1822,7 @@
         <v>62</v>
       </c>
       <c r="B68" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
NEW: Log Manager && Endgame UI Panel
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/Ending_String_Data.xlsx
+++ b/Assets/Internationalization/Ending_String_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\city_of_circling\city_of_circling\Assets\Internationalization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7847B7-679C-4BA5-B6B9-DB86E4576B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95077DA5-153B-4FBD-8A4A-4FEA8D908084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="1250" windowWidth="38620" windowHeight="21100" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4F4FC47A-7D6B-41F8-953F-5D527E753452}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
   <si>
     <t>key</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -743,6 +743,54 @@
       </rPr>
       <t>under the tree.</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LOG_COPY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LOG_COPIED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PLAY_AGAIN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>THANK_YOU</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Log Copied to Clipboard</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Play Again</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Copy Log</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>再次游玩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已复制到剪贴板</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>复制日志</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>感谢测试！\n为了更好地帮助我们设计，如您同意，请点击下方按钮导出游戏日志到您的剪贴板，并通过微信发送给我们。再次感谢！</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Thank you for playtesting! \nTo better help us design, if you agree, please click the button below to export the game log to your clipboard and send it to us through Discord. Much Appreciated!</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -814,7 +862,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -830,9 +878,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -870,7 +918,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -976,7 +1024,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1118,7 +1166,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1126,13 +1174,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E6B57D-D8BE-4224-A2B7-F664CEDC5AD4}">
-  <dimension ref="A1:C70"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:C74"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="24.08203125" customWidth="1"/>
+    <col min="1" max="1" width="24.125" customWidth="1"/>
     <col min="2" max="2" width="67.25" customWidth="1"/>
-    <col min="3" max="3" width="68.08203125" customWidth="1"/>
-    <col min="4" max="4" width="55.33203125" customWidth="1"/>
+    <col min="3" max="3" width="68.125" customWidth="1"/>
+    <col min="4" max="4" width="55.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1762,91 +1810,135 @@
         <v>54</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="42.75">
+      <c r="A62" t="s">
+        <v>198</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>195</v>
       </c>
       <c r="B63" t="s">
-        <v>78</v>
+        <v>201</v>
       </c>
       <c r="C63" t="s">
-        <v>66</v>
+        <v>204</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>58</v>
+        <v>196</v>
       </c>
       <c r="B64" t="s">
-        <v>168</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>184</v>
+        <v>199</v>
+      </c>
+      <c r="C64" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>59</v>
+        <v>197</v>
       </c>
       <c r="B65" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" t="s">
-        <v>60</v>
-      </c>
-      <c r="B66" t="s">
-        <v>77</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>68</v>
+        <v>200</v>
+      </c>
+      <c r="C65" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>76</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>70</v>
+        <v>78</v>
+      </c>
+      <c r="C67" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B68" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>73</v>
+        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B69" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>60</v>
+      </c>
+      <c r="B70" t="s">
+        <v>77</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>61</v>
+      </c>
+      <c r="B71" t="s">
+        <v>76</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>62</v>
+      </c>
+      <c r="B72" t="s">
+        <v>169</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>63</v>
+      </c>
+      <c r="B73" t="s">
+        <v>75</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
         <v>64</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B74" t="s">
         <v>74</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C74" s="1" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>